<commit_message>
Make generated resources cross-runtime deterministic
</commit_message>
<xml_diff>
--- a/assets/downloads/30-gunluk-denetim-hazirlik-plani-v1.xlsx
+++ b/assets/downloads/30-gunluk-denetim-hazirlik-plani-v1.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanım" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,17 +12,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Özet" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan'!$A$1:$H$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Özet'!$A$1:$B$4</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Plan'!$A$1:$H$31</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Özet'!$A$1:$B$4</definedName>
   </definedNames>
-  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="124519" calcMode="auto" forceFullCalc="1" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt formatCode="dd.mm.yyyy" numFmtId="164"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -119,39 +119,39 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="3" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="6" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="7" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -228,10 +228,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -387,7 +387,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -396,13 +396,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -412,7 +412,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dir="5400000" dist="20000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -421,7 +421,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dir="5400000" dist="23000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -430,7 +430,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dir="5400000" dist="23000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -440,12 +440,12 @@
             <a:camera prst="orthographicFront">
               <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
+            <a:lightRig dir="t" rig="threePt">
               <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
+            <a:bevelT h="25400" w="63500"/>
           </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
@@ -476,7 +476,7 @@
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+            <a:fillToRect b="180000" l="50000" r="50000" t="-80000"/>
           </a:path>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
@@ -495,7 +495,7 @@
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+            <a:fillToRect b="50000" l="50000" r="50000" t="50000"/>
           </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
@@ -515,8 +515,8 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col customWidth="1" max="1" min="1" width="26"/>
+    <col customWidth="1" max="2" min="2" width="70"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,7 +612,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -625,17 +625,17 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col customWidth="1" max="1" min="1" width="8"/>
+    <col customWidth="1" max="2" min="2" width="12"/>
+    <col customWidth="1" max="3" min="3" width="48"/>
+    <col customWidth="1" max="4" min="4" width="22"/>
+    <col customWidth="1" max="5" min="5" width="14"/>
+    <col customWidth="1" max="6" min="6" width="18"/>
+    <col customWidth="1" max="7" min="7" width="34"/>
+    <col customWidth="1" max="8" min="8" width="32"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row customHeight="1" ht="34" r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Gün</t>
@@ -1400,11 +1400,11 @@
   </sheetData>
   <autoFilter ref="A1:H31"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation allowBlank="0" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="F2:F31" type="list">
       <formula1>"Başlanmadı,Devam ediyor,Beklemede,Tamamlandı"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -1417,11 +1417,11 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col customWidth="1" max="1" min="1" width="28"/>
+    <col customWidth="1" max="2" min="2" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row customHeight="1" ht="34" r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Gösterge</t>
@@ -1468,6 +1468,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>